<commit_message>
Use AM demographics and same-APAC medications in third review outputs
- Take age and race/colour for Table 1 from AM fields (no missing values)
- Identify medications from AP_PRIPAL plus study medications dispensed within the same APAC (PA_QTDPRO > 0)
- Attribute doses and amounts to PA_PROC_ID, restricted to the eight study codes
- Clarify E22 as the ICD-10 category in the case-definition text
- Add medications_same_apac table and update Table 4, Figure 2 and medication tables
- Translate all third_review outputs to English
- Update third_review README and response draft
</commit_message>
<xml_diff>
--- a/resultados/third_review/20260907_acromegaly_annual_discontinuation.xlsx
+++ b/resultados/third_review/20260907_acromegaly_annual_discontinuation.xlsx
@@ -383,13 +383,13 @@
         </is>
       </c>
       <c r="B2">
-        <v>2021</v>
+        <v>2097</v>
       </c>
       <c r="C2">
-        <v>336</v>
+        <v>270</v>
       </c>
       <c r="D2">
-        <v>16.63</v>
+        <v>12.88</v>
       </c>
     </row>
     <row r="3">
@@ -399,13 +399,13 @@
         </is>
       </c>
       <c r="B3">
-        <v>900</v>
+        <v>1023</v>
       </c>
       <c r="C3">
-        <v>157</v>
+        <v>135</v>
       </c>
       <c r="D3">
-        <v>17.44</v>
+        <v>13.2</v>
       </c>
     </row>
     <row r="4">
@@ -415,13 +415,13 @@
         </is>
       </c>
       <c r="B4">
-        <v>814</v>
+        <v>976</v>
       </c>
       <c r="C4">
-        <v>157</v>
+        <v>105</v>
       </c>
       <c r="D4">
-        <v>19.29</v>
+        <v>10.76</v>
       </c>
     </row>
     <row r="5">
@@ -431,13 +431,13 @@
         </is>
       </c>
       <c r="B5">
-        <v>814</v>
+        <v>885</v>
       </c>
       <c r="C5">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="D5">
-        <v>15.97</v>
+        <v>14.8</v>
       </c>
     </row>
     <row r="6">
@@ -447,13 +447,13 @@
         </is>
       </c>
       <c r="B6">
-        <v>321</v>
+        <v>338</v>
       </c>
       <c r="C6">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D6">
-        <v>16.82</v>
+        <v>15.38</v>
       </c>
     </row>
     <row r="7">
@@ -463,13 +463,13 @@
         </is>
       </c>
       <c r="B7">
-        <v>87</v>
+        <v>94</v>
       </c>
       <c r="C7">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="D7">
-        <v>21.84</v>
+        <v>22.34</v>
       </c>
     </row>
     <row r="8">
@@ -479,13 +479,13 @@
         </is>
       </c>
       <c r="B8">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="C8">
         <v>7</v>
       </c>
       <c r="D8">
-        <v>14.29</v>
+        <v>12.96</v>
       </c>
     </row>
   </sheetData>

</xml_diff>